<commit_message>
docs: clean sensitive data, separate financial info to FINANZAS.md
</commit_message>
<xml_diff>
--- a/COMPARATIVA.xlsx
+++ b/COMPARATIVA.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>MGX offline editor. v2 = grupos. Pago 700+300€</t>
+          <t>MGX offline editor. v2 = grupos. Pago acuerdo</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>CFO propone 10.000€/año x 4h/día para grupos (NO concretado)</t>
+          <t>CFO propone acuerdo para grupos (NO concretado)</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Probable llamada: JMB cotiza 1.600€ y probablemente redefine alcance. Perfil Educativo → agrupaciones simples</t>
+          <t>Probable llamada: JMB cotiza acuerdo y probablemente redefine alcance. Perfil Educativo → agrupaciones simples</t>
         </is>
       </c>
     </row>
@@ -611,6 +611,8 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>

</xml_diff>